<commit_message>
Dedupe account-lockout bug (12-18 -> single #12); 17 bugs -> 12
Bugs 12,14-18 were identical except Role (now dropped per PDF spec).
Merged into one defect (all roles noted). Updated deck, README counts:
severity 8 low/4 medium, priority 3 high/5 medium/4 low.
</commit_message>
<xml_diff>
--- a/SauceDemo (Bug Report).xlsx
+++ b/SauceDemo (Bug Report).xlsx
@@ -94,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -121,6 +121,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -538,7 +544,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -577,7 +583,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -616,7 +622,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -656,7 +662,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -696,7 +702,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -738,7 +744,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -779,7 +785,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -820,7 +826,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>8</t>
         </is>
@@ -859,7 +865,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -897,7 +903,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
@@ -935,7 +941,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>11</t>
         </is>
@@ -974,7 +980,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>12</t>
         </is>
@@ -991,7 +997,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Account is not locked after multiple consecutive failed login attempts on Swag Labs login page</t>
+          <t>Account is not locked after multiple consecutive failed login attempts on Swag Labs login page — terjadi pada semua user role (standard, locked_out, problem, performance_glitch, error, visual).</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -1015,209 +1021,49 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Account is not locked after multiple consecutive failed login attempts on Swag Labs login page</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Account is not locked after multiple consecutive failed login attempts on Swag Labs login page</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Account is not locked after multiple consecutive failed login attempts on Swag Labs login page</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Account is not locked after multiple consecutive failed login attempts on Swag Labs login page</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="n"/>
+      <c r="G17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Account is not locked after multiple consecutive failed login attempts on Swag Labs login page</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>1. Go to "https://www.saucedemo.com/"
-2. Enter valid username
-3. Enter incorrect password 5 times
-4. Click Login</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>The system should display an error message, such as:
-"Epic sadface: Sorry, your account has been locked due to multiple failed login attempts. Please try again later."</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Epic sadface: Username and password do not match any user in this service</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>